<commit_message>
Semantic Review 02 - Begrippen A-B (vervolg)
</commit_message>
<xml_diff>
--- a/excel/Begrippenkader Beslag.xlsx
+++ b/excel/Begrippenkader Beslag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Mijn Documenten\GitHub\begrippenkader-beslag\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D25FF87-4DC0-4CAF-9D70-B72C162998CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFD7B2EC-3F1B-4978-8BE4-3555D9428547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="461">
   <si>
     <t>Titel</t>
   </si>
@@ -278,12 +278,15 @@
     <t>"Beslagbeslissing"@nl</t>
   </si>
   <si>
-    <t>"Een feitelijke beslissing over wat er (op grond van een bepaalde wettelijke bepaling) met een beslagvoorwerp moet gebeuren."@nl</t>
+    <t>"Beslissing waarbij wordt vastgesteld welke rechtsgevolgen voor een beslag of beslagvoorwerp worden toegepast."@nl</t>
   </si>
   <si>
     <t>"Er wordt niet gedifferentieerd naar beheerbeslissing en eindbeslissing, omdat in veel gevallen niet eenduidig is vast te stellen wanneer sprake is van een beheerbeslissing en wanneer van een eindbeslissing."@nl</t>
   </si>
   <si>
+    <t>ChatGPT – Semantic Review 02</t>
+  </si>
+  <si>
     <t>Begrip:Id-95443970-f0e1-d59b-5310-653015ad6b25</t>
   </si>
   <si>
@@ -356,7 +359,7 @@
     <t>"Beslaggebeurtenis"@nl</t>
   </si>
   <si>
-    <t>"Een handeling ten aanzien van een beslag."@nl</t>
+    <t>"Een activiteit die wordt uitgevoerd in het kader van het leggen, beheren of afwikkelen van strafvorderlijk beslag."@nl</t>
   </si>
   <si>
     <t>"Begrip:Id-20fbc366-da27-84cd-471d-3dc31d5b2818","Begrip:Id-7c43a980-a529-8d26-d9c5-46712970dd94"</t>
@@ -365,9 +368,6 @@
     <t>"Begrip:Id-4042164b-ee4b-7808-0ab1-842d69305d9d","Begrip:Id-60ca76c7-a48e-47b9-15ee-2fb9ad6c9f4b","Begrip:Id-654dfa9f-d10e-7b3c-eb67-2077adaad8be","Begrip:Id-d1b636df-f9ef-310c-cdf5-84b28a4b3478","Begrip:Id-dba51235-56a7-f9cd-6c98-80b3aff09f50","Begrip:Id-e2598bbe-bab5-f454-a722-c8379608d604"</t>
   </si>
   <si>
-    <t>"EB 2026-05-01: Bestaat er (al) een volledige lijst van alle voorkomende beslaghandelingen?"@nl</t>
-  </si>
-  <si>
     <t>Begrip:Id-7d991a97-eacd-e3b5-54d8-cf48bf53beb8</t>
   </si>
   <si>
@@ -383,7 +383,7 @@
     <t>"Beslagproces"@nl</t>
   </si>
   <si>
-    <t>"De verzameling van beslaghandelingen die heeft plaatsgevonden in de afhandeling van een beslag."@nl</t>
+    <t>"Het samenhangende geheel van beslaghandelingen dat wordt uitgevoerd vanaf het leggen tot en met de afwikkeling van een beslag."@nl</t>
   </si>
   <si>
     <t>"Begrip:Id-596dd23f-385d-aecd-fa46-d98a4e69a892","Begrip:Id-9717bcdf-19c1-a288-24a7-7ec01ae26b5c"</t>
@@ -392,7 +392,7 @@
     <t>"Beslagrol"@nl</t>
   </si>
   <si>
-    <t>"Een rol van een persoon ten aanzien van een beslag."@nl</t>
+    <t>"De verantwoordelijkheid of functie die een persoon of organisatie vervult binnen een beslagproces."@nl</t>
   </si>
   <si>
     <t>"Het begrip Persoon wordt hier gebruikt in de juridische zin, en kan daarom ook een rechtspersoon betreffen."@nl</t>
@@ -1350,6 +1350,9 @@
   </si>
   <si>
     <t>Besluitname</t>
+  </si>
+  <si>
+    <t>Definitie aangescherpt en proces/activiteit verduidelijkt.</t>
   </si>
   <si>
     <t>PROV</t>
@@ -1413,7 +1416,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1424,13 +1427,23 @@
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1450,9 +1463,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -2117,7 +2131,7 @@
       <c r="D11" t="s">
         <v>82</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="2" t="s">
         <v>83</v>
       </c>
       <c r="L11" t="s">
@@ -2126,13 +2140,13 @@
       <c r="AJ11" t="s">
         <v>48</v>
       </c>
-      <c r="AO11" t="s">
-        <v>64</v>
+      <c r="AO11" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
         <v>43</v>
@@ -2141,19 +2155,19 @@
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AJ12" t="s">
         <v>48</v>
       </c>
       <c r="AO12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.25">
@@ -2167,19 +2181,19 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R13" t="s">
         <v>71</v>
       </c>
       <c r="X13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AJ13" t="s">
         <v>48</v>
@@ -2190,7 +2204,7 @@
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
         <v>43</v>
@@ -2199,18 +2213,18 @@
         <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AO14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B15" t="s">
         <v>43</v>
@@ -2219,13 +2233,13 @@
         <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="W15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AJ15" t="s">
         <v>48</v>
@@ -2236,7 +2250,7 @@
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B16" t="s">
         <v>43</v>
@@ -2245,16 +2259,16 @@
         <v>44</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Q16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="R16" t="s">
         <v>71</v>
@@ -2268,7 +2282,7 @@
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B17" t="s">
         <v>43</v>
@@ -2277,28 +2291,28 @@
         <v>44</v>
       </c>
       <c r="D17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E17" t="s">
-        <v>108</v>
-      </c>
-      <c r="J17" t="s">
         <v>109</v>
       </c>
+      <c r="J17" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="M17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="X17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AJ17" t="s">
         <v>48</v>
       </c>
-      <c r="AO17" t="s">
-        <v>112</v>
+      <c r="AO17" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
@@ -2337,7 +2351,7 @@
       <c r="D19" t="s">
         <v>117</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="2" t="s">
         <v>118</v>
       </c>
       <c r="R19" t="s">
@@ -2346,10 +2360,13 @@
       <c r="AJ19" t="s">
         <v>48</v>
       </c>
+      <c r="AO19" s="2" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="20" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B20" t="s">
         <v>43</v>
@@ -2360,7 +2377,7 @@
       <c r="D20" t="s">
         <v>120</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="2" t="s">
         <v>121</v>
       </c>
       <c r="L20" t="s">
@@ -2371,6 +2388,9 @@
       </c>
       <c r="AJ20" t="s">
         <v>48</v>
+      </c>
+      <c r="AO20" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:41" x14ac:dyDescent="0.25">
@@ -2413,7 +2433,7 @@
         <v>130</v>
       </c>
       <c r="AO22" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
@@ -2488,7 +2508,7 @@
         <v>142</v>
       </c>
       <c r="W25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ25" t="s">
         <v>48</v>
@@ -2543,7 +2563,7 @@
         <v>48</v>
       </c>
       <c r="AO27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:41" x14ac:dyDescent="0.25">
@@ -2572,7 +2592,7 @@
         <v>48</v>
       </c>
       <c r="AO28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:41" x14ac:dyDescent="0.25">
@@ -2592,7 +2612,7 @@
         <v>157</v>
       </c>
       <c r="P29" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R29" t="s">
         <v>158</v>
@@ -2670,13 +2690,13 @@
         <v>170</v>
       </c>
       <c r="W32" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AJ32" t="s">
         <v>48</v>
       </c>
       <c r="AO32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:41" x14ac:dyDescent="0.25">
@@ -2702,7 +2722,7 @@
         <v>48</v>
       </c>
       <c r="AO33" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:41" x14ac:dyDescent="0.25">
@@ -2797,7 +2817,7 @@
         <v>188</v>
       </c>
       <c r="W37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ37" t="s">
         <v>48</v>
@@ -2849,7 +2869,7 @@
         <v>48</v>
       </c>
       <c r="AO39" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:41" x14ac:dyDescent="0.25">
@@ -2901,7 +2921,7 @@
         <v>48</v>
       </c>
       <c r="AO41" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" spans="1:41" x14ac:dyDescent="0.25">
@@ -2930,7 +2950,7 @@
         <v>48</v>
       </c>
       <c r="AO42" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:41" x14ac:dyDescent="0.25">
@@ -3082,7 +3102,7 @@
         <v>225</v>
       </c>
       <c r="P49" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R49" t="s">
         <v>155</v>
@@ -3134,7 +3154,7 @@
         <v>48</v>
       </c>
       <c r="AO51" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:41" x14ac:dyDescent="0.25">
@@ -3232,7 +3252,7 @@
         <v>245</v>
       </c>
       <c r="AO55" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="56" spans="1:41" x14ac:dyDescent="0.25">
@@ -3321,7 +3341,7 @@
         <v>257</v>
       </c>
       <c r="AO59" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:41" x14ac:dyDescent="0.25">
@@ -3603,7 +3623,7 @@
         <v>296</v>
       </c>
       <c r="W71" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AJ71" t="s">
         <v>48</v>
@@ -3661,7 +3681,7 @@
         <v>48</v>
       </c>
       <c r="AO73" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="74" spans="1:41" x14ac:dyDescent="0.25">
@@ -3779,7 +3799,7 @@
         <v>316</v>
       </c>
       <c r="L78" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="AJ78" t="s">
         <v>48</v>
@@ -3877,7 +3897,7 @@
         <v>328</v>
       </c>
       <c r="R82" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ82" t="s">
         <v>48</v>
@@ -4067,7 +4087,7 @@
         <v>353</v>
       </c>
       <c r="W90" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ90" t="s">
         <v>48</v>
@@ -4116,7 +4136,7 @@
         <v>359</v>
       </c>
       <c r="W92" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ92" t="s">
         <v>48</v>
@@ -4191,7 +4211,7 @@
         <v>48</v>
       </c>
       <c r="AO95" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="1:41" x14ac:dyDescent="0.25">
@@ -4286,7 +4306,7 @@
         <v>375</v>
       </c>
       <c r="W99" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ99" t="s">
         <v>48</v>
@@ -4381,7 +4401,7 @@
         <v>392</v>
       </c>
       <c r="W103" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AJ103" t="s">
         <v>48</v>
@@ -4522,7 +4542,7 @@
         <v>410</v>
       </c>
       <c r="L109" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R109" t="s">
         <v>411</v>
@@ -4534,7 +4554,7 @@
         <v>48</v>
       </c>
       <c r="AO109" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="110" spans="1:41" x14ac:dyDescent="0.25">
@@ -4688,7 +4708,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -4733,6 +4753,50 @@
       </c>
       <c r="C4" t="s">
         <v>438</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" t="s">
+        <v>437</v>
+      </c>
+      <c r="C5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" t="s">
+        <v>437</v>
+      </c>
+      <c r="C6" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" t="s">
+        <v>437</v>
+      </c>
+      <c r="C7" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" t="s">
+        <v>437</v>
+      </c>
+      <c r="C8" t="s">
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -4753,7 +4817,7 @@
         <v>434</v>
       </c>
       <c r="C1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4761,10 +4825,10 @@
         <v>436</v>
       </c>
       <c r="B2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4772,10 +4836,10 @@
         <v>439</v>
       </c>
       <c r="B3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C3" t="s">
         <v>444</v>
-      </c>
-      <c r="C3" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4783,87 +4847,87 @@
         <v>440</v>
       </c>
       <c r="B4" t="s">
+        <v>445</v>
+      </c>
+      <c r="C4" t="s">
         <v>444</v>
-      </c>
-      <c r="C4" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>449</v>
+      </c>
+      <c r="B6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" t="s">
         <v>448</v>
-      </c>
-      <c r="B6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C6" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B8" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C8" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>456</v>
+      </c>
+      <c r="B9" t="s">
+        <v>457</v>
+      </c>
+      <c r="C9" t="s">
         <v>455</v>
-      </c>
-      <c r="B9" t="s">
-        <v>456</v>
-      </c>
-      <c r="C9" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B10" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C10" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>460</v>
+      </c>
+      <c r="B11" t="s">
         <v>459</v>
       </c>
-      <c r="B11" t="s">
-        <v>458</v>
-      </c>
       <c r="C11" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Opschoning uitgevoerd op tabbladen Redactieoverzicht en Begripstypering. Inhoud van CHANGELOG.md teruggebracht tot enkel een inleidend stukje tekst. Dit nadat was gebleken dat er discrepanties bestonden tussen wat als wijzigingen was beschreven en wat er daadwerkelijk was aangepast in de Excel-sheet.
</commit_message>
<xml_diff>
--- a/excel/Begrippenkader Beslag.xlsx
+++ b/excel/Begrippenkader Beslag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Mijn Documenten\GitHub\begrippenkader-beslag\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFD7B2EC-3F1B-4978-8BE4-3555D9428547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A77FE9-6264-4885-91CD-FA3D8397C23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="437">
   <si>
     <t>Titel</t>
   </si>
@@ -239,9 +239,6 @@
     <t>"Beslag bewaring"@nl</t>
   </si>
   <si>
-    <t>Het bewaren van een beslagvoorwerp gedurende de periode waarin daarop strafvorderlijk beslag rust.</t>
-  </si>
-  <si>
     <t>Begrip:Id-0c79c3d8-bdd3-b152-fa07-ac4cad6f33a7</t>
   </si>
   <si>
@@ -1337,86 +1334,17 @@
     <t>Toelichting</t>
   </si>
   <si>
-    <t>Beslag beheer</t>
-  </si>
-  <si>
-    <t>Inhoudelijk</t>
-  </si>
-  <si>
-    <t>Definitie aangescherpt.</t>
-  </si>
-  <si>
-    <t>Beslag bewaring</t>
-  </si>
-  <si>
-    <t>Besluitname</t>
-  </si>
-  <si>
-    <t>Definitie aangescherpt en proces/activiteit verduidelijkt.</t>
-  </si>
-  <si>
     <t>PROV</t>
   </si>
   <si>
-    <t>Proces</t>
-  </si>
-  <si>
-    <t>Activity</t>
-  </si>
-  <si>
-    <t>Activiteit</t>
-  </si>
-  <si>
-    <t>Beslagbeheerder</t>
-  </si>
-  <si>
-    <t>Rol</t>
-  </si>
-  <si>
-    <t>Agent</t>
-  </si>
-  <si>
-    <t>Beslagbewaarder</t>
-  </si>
-  <si>
-    <t>Beslagportaal</t>
-  </si>
-  <si>
-    <t>Informatiesysteem</t>
-  </si>
-  <si>
-    <t>Agent?</t>
-  </si>
-  <si>
-    <t>Beslagvoorwerp</t>
-  </si>
-  <si>
-    <t>Voorwerp</t>
-  </si>
-  <si>
-    <t>Entity</t>
-  </si>
-  <si>
-    <t>Beslagzaak</t>
-  </si>
-  <si>
-    <t>Zaak</t>
-  </si>
-  <si>
-    <t>Beslag</t>
-  </si>
-  <si>
-    <t>Juridisch begrip</t>
-  </si>
-  <si>
-    <t>Beslagbeslissing</t>
+    <t>"Het bewaren van een beslagvoorwerp gedurende de periode waarin daarop strafvorderlijk beslag rust."@nl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1431,6 +1359,23 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1460,15 +1405,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1773,6 +1723,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AP115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="9.140625" style="4"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1802,7 +1755,7 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="K1" t="s">
@@ -1915,7 +1868,7 @@
       <c r="D2" t="s">
         <v>45</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="4" t="s">
         <v>46</v>
       </c>
       <c r="W2" t="s">
@@ -1941,7 +1894,7 @@
       <c r="D3" t="s">
         <v>51</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="4" t="s">
         <v>52</v>
       </c>
       <c r="W3" t="s">
@@ -1967,7 +1920,7 @@
       <c r="D4" t="s">
         <v>54</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="4" t="s">
         <v>55</v>
       </c>
       <c r="AJ4" t="s">
@@ -1987,7 +1940,7 @@
       <c r="D5" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="4" t="s">
         <v>58</v>
       </c>
       <c r="AJ5" t="s">
@@ -2010,7 +1963,7 @@
       <c r="D6" t="s">
         <v>61</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="4" t="s">
         <v>62</v>
       </c>
       <c r="P6" t="s">
@@ -2036,7 +1989,7 @@
       <c r="D7" t="s">
         <v>66</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="4" t="s">
         <v>67</v>
       </c>
       <c r="AJ7" t="s">
@@ -2056,8 +2009,8 @@
       <c r="D8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>70</v>
+      <c r="J8" s="3" t="s">
+        <v>436</v>
       </c>
       <c r="AJ8" t="s">
         <v>48</v>
@@ -2068,106 +2021,106 @@
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
         <v>71</v>
       </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="J9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="J9" t="s">
+      <c r="R9" t="s">
         <v>73</v>
       </c>
-      <c r="R9" t="s">
+      <c r="T9" t="s">
         <v>74</v>
       </c>
-      <c r="T9" t="s">
+      <c r="AJ9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO9" t="s">
         <v>75</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
         <v>77</v>
       </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="J10" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="J10" t="s">
+      <c r="AJ10" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO10" t="s">
         <v>79</v>
-      </c>
-      <c r="AJ10" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
         <v>81</v>
       </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="J11" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="L11" t="s">
         <v>83</v>
       </c>
-      <c r="L11" t="s">
+      <c r="AJ11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO11" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO11" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
         <v>86</v>
       </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="J12" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="J12" t="s">
+      <c r="L12" t="s">
         <v>88</v>
       </c>
-      <c r="L12" t="s">
+      <c r="AJ12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO12" t="s">
         <v>89</v>
-      </c>
-      <c r="AJ12" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO12" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.25">
@@ -2181,65 +2134,65 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
+        <v>90</v>
+      </c>
+      <c r="J13" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="J13" t="s">
+      <c r="L13" t="s">
+        <v>88</v>
+      </c>
+      <c r="R13" t="s">
+        <v>70</v>
+      </c>
+      <c r="X13" t="s">
         <v>92</v>
       </c>
-      <c r="L13" t="s">
-        <v>89</v>
-      </c>
-      <c r="R13" t="s">
-        <v>71</v>
-      </c>
-      <c r="X13" t="s">
-        <v>93</v>
-      </c>
       <c r="AJ13" t="s">
         <v>48</v>
       </c>
       <c r="AO13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
         <v>94</v>
       </c>
-      <c r="B14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="J14" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="J14" t="s">
+      <c r="AO14" t="s">
         <v>96</v>
-      </c>
-      <c r="AO14" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
         <v>98</v>
       </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="J15" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J15" t="s">
+      <c r="W15" t="s">
         <v>100</v>
-      </c>
-      <c r="W15" t="s">
-        <v>101</v>
       </c>
       <c r="AJ15" t="s">
         <v>48</v>
@@ -2250,123 +2203,123 @@
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
         <v>102</v>
       </c>
-      <c r="B16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>103</v>
       </c>
-      <c r="E16" t="s">
+      <c r="J16" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="J16" t="s">
+      <c r="Q16" t="s">
         <v>105</v>
       </c>
-      <c r="Q16" t="s">
-        <v>106</v>
-      </c>
       <c r="R16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AJ16" t="s">
         <v>48</v>
       </c>
       <c r="AO16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
         <v>107</v>
       </c>
-      <c r="B17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>108</v>
       </c>
-      <c r="E17" t="s">
+      <c r="J17" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="M17" t="s">
+        <v>88</v>
+      </c>
+      <c r="R17" t="s">
         <v>110</v>
       </c>
-      <c r="M17" t="s">
-        <v>89</v>
-      </c>
-      <c r="R17" t="s">
+      <c r="X17" t="s">
         <v>111</v>
       </c>
-      <c r="X17" t="s">
-        <v>112</v>
-      </c>
       <c r="AJ17" t="s">
         <v>48</v>
       </c>
       <c r="AO17" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
         <v>113</v>
       </c>
-      <c r="B18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="J18" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="J18" t="s">
-        <v>115</v>
-      </c>
       <c r="AJ18" t="s">
         <v>48</v>
       </c>
       <c r="AO18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
         <v>116</v>
       </c>
-      <c r="B19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="J19" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="R19" t="s">
         <v>118</v>
       </c>
-      <c r="R19" t="s">
-        <v>119</v>
-      </c>
       <c r="AJ19" t="s">
         <v>48</v>
       </c>
       <c r="AO19" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
         <v>43</v>
@@ -2375,163 +2328,163 @@
         <v>44</v>
       </c>
       <c r="D20" t="s">
+        <v>119</v>
+      </c>
+      <c r="J20" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="L20" t="s">
         <v>121</v>
       </c>
-      <c r="L20" t="s">
+      <c r="X20" t="s">
         <v>122</v>
       </c>
-      <c r="X20" t="s">
-        <v>123</v>
-      </c>
       <c r="AJ20" t="s">
         <v>48</v>
       </c>
       <c r="AO20" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
         <v>124</v>
       </c>
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="J21" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="J21" t="s">
+      <c r="AJ21" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO21" t="s">
         <v>126</v>
-      </c>
-      <c r="AJ21" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO21" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
         <v>128</v>
       </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="J22" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="J22" t="s">
-        <v>130</v>
-      </c>
       <c r="AO22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
         <v>131</v>
       </c>
-      <c r="B23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>132</v>
       </c>
-      <c r="E23" t="s">
+      <c r="J23" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="J23" t="s">
+      <c r="L23" t="s">
         <v>134</v>
       </c>
-      <c r="L23" t="s">
-        <v>135</v>
-      </c>
       <c r="AJ23" t="s">
         <v>48</v>
       </c>
       <c r="AO23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
         <v>136</v>
       </c>
-      <c r="B24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="J24" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="J24" t="s">
-        <v>138</v>
-      </c>
       <c r="AJ24" t="s">
         <v>48</v>
       </c>
       <c r="AO24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
         <v>139</v>
       </c>
-      <c r="B25" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>140</v>
       </c>
-      <c r="E25" t="s">
+      <c r="J25" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="J25" t="s">
+      <c r="W25" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO25" t="s">
         <v>142</v>
-      </c>
-      <c r="W25" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ25" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO25" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>143</v>
+      </c>
+      <c r="B26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
         <v>144</v>
       </c>
-      <c r="B26" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" t="s">
-        <v>44</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="J26" s="4" t="s">
         <v>145</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="AJ26" t="s">
         <v>48</v>
@@ -2542,80 +2495,80 @@
     </row>
     <row r="27" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s">
         <v>147</v>
       </c>
-      <c r="B27" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="J27" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="J27" t="s">
+      <c r="L27" t="s">
         <v>149</v>
       </c>
-      <c r="L27" t="s">
-        <v>150</v>
-      </c>
       <c r="AJ27" t="s">
         <v>48</v>
       </c>
       <c r="AO27" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
         <v>151</v>
       </c>
-      <c r="B28" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="J28" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="J28" t="s">
+      <c r="R28" t="s">
         <v>153</v>
       </c>
-      <c r="R28" t="s">
-        <v>154</v>
-      </c>
       <c r="S28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AJ28" t="s">
         <v>48</v>
       </c>
       <c r="AO28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>154</v>
+      </c>
+      <c r="B29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" t="s">
         <v>155</v>
       </c>
-      <c r="B29" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="J29" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="J29" t="s">
+      <c r="P29" t="s">
+        <v>101</v>
+      </c>
+      <c r="R29" t="s">
         <v>157</v>
-      </c>
-      <c r="P29" t="s">
-        <v>102</v>
-      </c>
-      <c r="R29" t="s">
-        <v>158</v>
       </c>
       <c r="AJ29" t="s">
         <v>48</v>
@@ -2623,126 +2576,126 @@
     </row>
     <row r="30" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" t="s">
         <v>159</v>
       </c>
-      <c r="B30" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="J30" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J30" t="s">
-        <v>161</v>
-      </c>
       <c r="AJ30" t="s">
         <v>48</v>
       </c>
       <c r="AO30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" t="s">
         <v>162</v>
       </c>
-      <c r="B31" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="J31" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="J31" t="s">
+      <c r="L31" t="s">
         <v>164</v>
       </c>
-      <c r="L31" t="s">
+      <c r="S31" t="s">
         <v>165</v>
       </c>
-      <c r="S31" t="s">
+      <c r="AJ31" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO31" t="s">
         <v>166</v>
-      </c>
-      <c r="AJ31" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO31" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="32" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>167</v>
+      </c>
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
         <v>168</v>
       </c>
-      <c r="B32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="J32" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="J32" t="s">
-        <v>170</v>
-      </c>
       <c r="W32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AJ32" t="s">
         <v>48</v>
       </c>
       <c r="AO32" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
         <v>171</v>
       </c>
-      <c r="B33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="J33" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="J33" t="s">
+      <c r="S33" t="s">
         <v>173</v>
       </c>
-      <c r="S33" t="s">
-        <v>174</v>
-      </c>
       <c r="AJ33" t="s">
         <v>48</v>
       </c>
       <c r="AO33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>174</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" t="s">
         <v>175</v>
       </c>
-      <c r="B34" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="J34" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="J34" t="s">
+      <c r="P34" t="s">
         <v>177</v>
-      </c>
-      <c r="P34" t="s">
-        <v>178</v>
       </c>
       <c r="AJ34" t="s">
         <v>48</v>
@@ -2753,48 +2706,48 @@
     </row>
     <row r="35" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" t="s">
         <v>179</v>
       </c>
-      <c r="B35" t="s">
-        <v>43</v>
-      </c>
-      <c r="C35" t="s">
-        <v>44</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="J35" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="J35" t="s">
-        <v>181</v>
-      </c>
       <c r="AJ35" t="s">
         <v>48</v>
       </c>
       <c r="AO35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>181</v>
+      </c>
+      <c r="B36" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" t="s">
         <v>182</v>
       </c>
-      <c r="B36" t="s">
-        <v>43</v>
-      </c>
-      <c r="C36" t="s">
-        <v>44</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="J36" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="J36" t="s">
+      <c r="L36" t="s">
         <v>184</v>
       </c>
-      <c r="L36" t="s">
-        <v>185</v>
-      </c>
       <c r="R36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AJ36" t="s">
         <v>48</v>
@@ -2802,22 +2755,22 @@
     </row>
     <row r="37" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>185</v>
+      </c>
+      <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" t="s">
         <v>186</v>
       </c>
-      <c r="B37" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" t="s">
-        <v>44</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="J37" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="J37" t="s">
-        <v>188</v>
-      </c>
       <c r="W37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AJ37" t="s">
         <v>48</v>
@@ -2828,19 +2781,19 @@
     </row>
     <row r="38" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>188</v>
+      </c>
+      <c r="B38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" t="s">
         <v>189</v>
       </c>
-      <c r="B38" t="s">
-        <v>43</v>
-      </c>
-      <c r="C38" t="s">
-        <v>44</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="J38" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="J38" t="s">
-        <v>191</v>
       </c>
       <c r="AJ38" t="s">
         <v>48</v>
@@ -2848,56 +2801,56 @@
     </row>
     <row r="39" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>191</v>
+      </c>
+      <c r="B39" t="s">
+        <v>43</v>
+      </c>
+      <c r="C39" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" t="s">
         <v>192</v>
       </c>
-      <c r="B39" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" t="s">
-        <v>44</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>193</v>
       </c>
-      <c r="E39" t="s">
+      <c r="J39" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="J39" t="s">
-        <v>195</v>
-      </c>
       <c r="AJ39" t="s">
         <v>48</v>
       </c>
       <c r="AO39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>195</v>
+      </c>
+      <c r="B40" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" t="s">
+        <v>44</v>
+      </c>
+      <c r="D40" t="s">
         <v>196</v>
       </c>
-      <c r="B40" t="s">
-        <v>43</v>
-      </c>
-      <c r="C40" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="J40" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="J40" t="s">
-        <v>198</v>
-      </c>
       <c r="AJ40" t="s">
         <v>48</v>
       </c>
       <c r="AO40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B41" t="s">
         <v>43</v>
@@ -2906,91 +2859,91 @@
         <v>44</v>
       </c>
       <c r="D41" t="s">
+        <v>198</v>
+      </c>
+      <c r="J41" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="J41" t="s">
-        <v>200</v>
-      </c>
       <c r="R41" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="S41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AJ41" t="s">
         <v>48</v>
       </c>
       <c r="AO41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="42" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>200</v>
+      </c>
+      <c r="B42" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" t="s">
+        <v>44</v>
+      </c>
+      <c r="D42" t="s">
         <v>201</v>
       </c>
-      <c r="B42" t="s">
-        <v>43</v>
-      </c>
-      <c r="C42" t="s">
-        <v>44</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="F42" t="s">
         <v>202</v>
       </c>
-      <c r="F42" t="s">
+      <c r="J42" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="J42" t="s">
+      <c r="L42" t="s">
         <v>204</v>
       </c>
-      <c r="L42" t="s">
-        <v>205</v>
-      </c>
       <c r="AJ42" t="s">
         <v>48</v>
       </c>
       <c r="AO42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>205</v>
+      </c>
+      <c r="B43" t="s">
+        <v>43</v>
+      </c>
+      <c r="C43" t="s">
+        <v>44</v>
+      </c>
+      <c r="D43" t="s">
         <v>206</v>
       </c>
-      <c r="B43" t="s">
-        <v>43</v>
-      </c>
-      <c r="C43" t="s">
-        <v>44</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="J43" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="J43" t="s">
-        <v>208</v>
-      </c>
       <c r="AJ43" t="s">
         <v>48</v>
       </c>
       <c r="AO43" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>208</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
         <v>209</v>
       </c>
-      <c r="B44" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" t="s">
-        <v>44</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="J44" s="4" t="s">
         <v>210</v>
-      </c>
-      <c r="J44" t="s">
-        <v>211</v>
       </c>
       <c r="AJ44" t="s">
         <v>48</v>
@@ -2998,88 +2951,88 @@
     </row>
     <row r="45" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>211</v>
+      </c>
+      <c r="B45" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
         <v>212</v>
       </c>
-      <c r="B45" t="s">
-        <v>43</v>
-      </c>
-      <c r="C45" t="s">
-        <v>44</v>
-      </c>
-      <c r="D45" t="s">
+      <c r="J45" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="J45" t="s">
-        <v>214</v>
-      </c>
       <c r="AJ45" t="s">
         <v>48</v>
       </c>
       <c r="AO45" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>214</v>
+      </c>
+      <c r="B46" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
         <v>215</v>
       </c>
-      <c r="B46" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="J46" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="J46" t="s">
-        <v>217</v>
-      </c>
       <c r="AJ46" t="s">
         <v>48</v>
       </c>
       <c r="AO46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>217</v>
+      </c>
+      <c r="B47" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" t="s">
         <v>218</v>
       </c>
-      <c r="B47" t="s">
-        <v>43</v>
-      </c>
-      <c r="C47" t="s">
-        <v>44</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="J47" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="J47" t="s">
-        <v>220</v>
-      </c>
       <c r="AJ47" t="s">
         <v>48</v>
       </c>
       <c r="AO47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>220</v>
+      </c>
+      <c r="B48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" t="s">
         <v>221</v>
       </c>
-      <c r="B48" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" t="s">
-        <v>44</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="J48" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="J48" t="s">
-        <v>223</v>
       </c>
       <c r="AJ48" t="s">
         <v>48</v>
@@ -3087,7 +3040,7 @@
     </row>
     <row r="49" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B49" t="s">
         <v>43</v>
@@ -3096,16 +3049,16 @@
         <v>44</v>
       </c>
       <c r="D49" t="s">
+        <v>223</v>
+      </c>
+      <c r="J49" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="J49" t="s">
-        <v>225</v>
-      </c>
       <c r="P49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="R49" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AJ49" t="s">
         <v>48</v>
@@ -3122,10 +3075,10 @@
         <v>44</v>
       </c>
       <c r="D50" t="s">
+        <v>225</v>
+      </c>
+      <c r="J50" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="J50" t="s">
-        <v>227</v>
       </c>
       <c r="Q50" t="s">
         <v>60</v>
@@ -3136,48 +3089,48 @@
     </row>
     <row r="51" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>227</v>
+      </c>
+      <c r="B51" t="s">
+        <v>43</v>
+      </c>
+      <c r="C51" t="s">
+        <v>44</v>
+      </c>
+      <c r="D51" t="s">
         <v>228</v>
       </c>
-      <c r="B51" t="s">
-        <v>43</v>
-      </c>
-      <c r="C51" t="s">
-        <v>44</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="J51" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="J51" t="s">
-        <v>230</v>
-      </c>
       <c r="AJ51" t="s">
         <v>48</v>
       </c>
       <c r="AO51" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="52" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>230</v>
+      </c>
+      <c r="B52" t="s">
+        <v>43</v>
+      </c>
+      <c r="C52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D52" t="s">
         <v>231</v>
       </c>
-      <c r="B52" t="s">
-        <v>43</v>
-      </c>
-      <c r="C52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="G52" t="s">
         <v>232</v>
       </c>
-      <c r="G52" t="s">
+      <c r="J52" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="J52" t="s">
-        <v>234</v>
-      </c>
       <c r="S52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AJ52" t="s">
         <v>48</v>
@@ -3185,255 +3138,255 @@
     </row>
     <row r="53" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>234</v>
+      </c>
+      <c r="B53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C53" t="s">
+        <v>44</v>
+      </c>
+      <c r="D53" t="s">
         <v>235</v>
       </c>
-      <c r="B53" t="s">
-        <v>43</v>
-      </c>
-      <c r="C53" t="s">
-        <v>44</v>
-      </c>
-      <c r="D53" t="s">
+      <c r="J53" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="J53" t="s">
+      <c r="R53" t="s">
         <v>237</v>
       </c>
-      <c r="R53" t="s">
+      <c r="S53" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ53" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO53" t="s">
         <v>238</v>
-      </c>
-      <c r="S53" t="s">
-        <v>166</v>
-      </c>
-      <c r="AJ53" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO53" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="54" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>239</v>
+      </c>
+      <c r="B54" t="s">
+        <v>43</v>
+      </c>
+      <c r="C54" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54" t="s">
         <v>240</v>
       </c>
-      <c r="B54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C54" t="s">
-        <v>44</v>
-      </c>
-      <c r="D54" t="s">
+      <c r="J54" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="J54" t="s">
-        <v>242</v>
-      </c>
       <c r="AJ54" t="s">
         <v>48</v>
       </c>
       <c r="AO54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>242</v>
+      </c>
+      <c r="B55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55" t="s">
+        <v>44</v>
+      </c>
+      <c r="D55" t="s">
         <v>243</v>
       </c>
-      <c r="B55" t="s">
-        <v>43</v>
-      </c>
-      <c r="C55" t="s">
-        <v>44</v>
-      </c>
-      <c r="D55" t="s">
+      <c r="J55" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="J55" t="s">
-        <v>245</v>
-      </c>
       <c r="AO55" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>245</v>
+      </c>
+      <c r="B56" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" t="s">
+        <v>44</v>
+      </c>
+      <c r="D56" t="s">
         <v>246</v>
       </c>
-      <c r="B56" t="s">
-        <v>43</v>
-      </c>
-      <c r="C56" t="s">
-        <v>44</v>
-      </c>
-      <c r="D56" t="s">
+      <c r="J56" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="J56" t="s">
-        <v>248</v>
-      </c>
       <c r="AJ56" t="s">
         <v>48</v>
       </c>
       <c r="AO56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>248</v>
+      </c>
+      <c r="B57" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" t="s">
+        <v>44</v>
+      </c>
+      <c r="D57" t="s">
         <v>249</v>
       </c>
-      <c r="B57" t="s">
-        <v>43</v>
-      </c>
-      <c r="C57" t="s">
-        <v>44</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="J57" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="J57" t="s">
-        <v>251</v>
-      </c>
       <c r="AJ57" t="s">
         <v>48</v>
       </c>
       <c r="AO57" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>251</v>
+      </c>
+      <c r="B58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" t="s">
+        <v>44</v>
+      </c>
+      <c r="D58" t="s">
         <v>252</v>
       </c>
-      <c r="B58" t="s">
-        <v>43</v>
-      </c>
-      <c r="C58" t="s">
-        <v>44</v>
-      </c>
-      <c r="D58" t="s">
+      <c r="J58" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="J58" t="s">
-        <v>254</v>
-      </c>
       <c r="AJ58" t="s">
         <v>48</v>
       </c>
       <c r="AO58" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>254</v>
+      </c>
+      <c r="B59" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" t="s">
+        <v>44</v>
+      </c>
+      <c r="D59" t="s">
         <v>255</v>
       </c>
-      <c r="B59" t="s">
-        <v>43</v>
-      </c>
-      <c r="C59" t="s">
-        <v>44</v>
-      </c>
-      <c r="D59" t="s">
+      <c r="J59" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="J59" t="s">
-        <v>257</v>
-      </c>
       <c r="AO59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>257</v>
+      </c>
+      <c r="B60" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" t="s">
+        <v>44</v>
+      </c>
+      <c r="D60" t="s">
         <v>258</v>
       </c>
-      <c r="B60" t="s">
-        <v>43</v>
-      </c>
-      <c r="C60" t="s">
-        <v>44</v>
-      </c>
-      <c r="D60" t="s">
+      <c r="J60" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="J60" t="s">
-        <v>260</v>
-      </c>
       <c r="AJ60" t="s">
         <v>48</v>
       </c>
       <c r="AO60" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="61" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>260</v>
+      </c>
+      <c r="B61" t="s">
+        <v>43</v>
+      </c>
+      <c r="C61" t="s">
+        <v>44</v>
+      </c>
+      <c r="D61" t="s">
         <v>261</v>
       </c>
-      <c r="B61" t="s">
-        <v>43</v>
-      </c>
-      <c r="C61" t="s">
-        <v>44</v>
-      </c>
-      <c r="D61" t="s">
+      <c r="J61" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="J61" t="s">
+      <c r="S61" t="s">
+        <v>173</v>
+      </c>
+      <c r="AJ61" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO61" t="s">
         <v>263</v>
-      </c>
-      <c r="S61" t="s">
-        <v>174</v>
-      </c>
-      <c r="AJ61" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO61" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="62" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>264</v>
+      </c>
+      <c r="B62" t="s">
+        <v>43</v>
+      </c>
+      <c r="C62" t="s">
+        <v>44</v>
+      </c>
+      <c r="D62" t="s">
         <v>265</v>
       </c>
-      <c r="B62" t="s">
-        <v>43</v>
-      </c>
-      <c r="C62" t="s">
-        <v>44</v>
-      </c>
-      <c r="D62" t="s">
+      <c r="J62" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="J62" t="s">
+      <c r="S62" t="s">
         <v>267</v>
       </c>
-      <c r="S62" t="s">
+      <c r="AJ62" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO62" t="s">
         <v>268</v>
-      </c>
-      <c r="AJ62" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO62" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>269</v>
+      </c>
+      <c r="B63" t="s">
+        <v>43</v>
+      </c>
+      <c r="C63" t="s">
+        <v>44</v>
+      </c>
+      <c r="D63" t="s">
         <v>270</v>
       </c>
-      <c r="B63" t="s">
-        <v>43</v>
-      </c>
-      <c r="C63" t="s">
-        <v>44</v>
-      </c>
-      <c r="D63" t="s">
+      <c r="J63" s="4" t="s">
         <v>271</v>
-      </c>
-      <c r="J63" t="s">
-        <v>272</v>
       </c>
       <c r="AJ63" t="s">
         <v>48</v>
@@ -3444,88 +3397,88 @@
     </row>
     <row r="64" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>272</v>
+      </c>
+      <c r="B64" t="s">
+        <v>43</v>
+      </c>
+      <c r="C64" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" t="s">
         <v>273</v>
       </c>
-      <c r="B64" t="s">
-        <v>43</v>
-      </c>
-      <c r="C64" t="s">
-        <v>44</v>
-      </c>
-      <c r="D64" t="s">
+      <c r="J64" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="J64" t="s">
-        <v>275</v>
-      </c>
       <c r="AJ64" t="s">
         <v>48</v>
       </c>
       <c r="AO64" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="65" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>275</v>
+      </c>
+      <c r="B65" t="s">
+        <v>43</v>
+      </c>
+      <c r="C65" t="s">
+        <v>44</v>
+      </c>
+      <c r="D65" t="s">
         <v>276</v>
       </c>
-      <c r="B65" t="s">
-        <v>43</v>
-      </c>
-      <c r="C65" t="s">
-        <v>44</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="J65" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="J65" t="s">
-        <v>278</v>
-      </c>
       <c r="AJ65" t="s">
         <v>48</v>
       </c>
       <c r="AO65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>278</v>
+      </c>
+      <c r="B66" t="s">
+        <v>43</v>
+      </c>
+      <c r="C66" t="s">
+        <v>44</v>
+      </c>
+      <c r="D66" t="s">
         <v>279</v>
       </c>
-      <c r="B66" t="s">
-        <v>43</v>
-      </c>
-      <c r="C66" t="s">
-        <v>44</v>
-      </c>
-      <c r="D66" t="s">
+      <c r="J66" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="J66" t="s">
-        <v>281</v>
-      </c>
       <c r="AJ66" t="s">
         <v>48</v>
       </c>
       <c r="AO66" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>281</v>
+      </c>
+      <c r="B67" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" t="s">
+        <v>44</v>
+      </c>
+      <c r="D67" t="s">
         <v>282</v>
       </c>
-      <c r="B67" t="s">
-        <v>43</v>
-      </c>
-      <c r="C67" t="s">
-        <v>44</v>
-      </c>
-      <c r="D67" t="s">
+      <c r="J67" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="J67" t="s">
-        <v>284</v>
       </c>
       <c r="AJ67" t="s">
         <v>48</v>
@@ -3536,7 +3489,7 @@
     </row>
     <row r="68" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B68" t="s">
         <v>43</v>
@@ -3545,16 +3498,16 @@
         <v>44</v>
       </c>
       <c r="D68" t="s">
+        <v>284</v>
+      </c>
+      <c r="J68" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="J68" t="s">
+      <c r="Q68" t="s">
+        <v>174</v>
+      </c>
+      <c r="T68" t="s">
         <v>286</v>
-      </c>
-      <c r="Q68" t="s">
-        <v>175</v>
-      </c>
-      <c r="T68" t="s">
-        <v>287</v>
       </c>
       <c r="AJ68" t="s">
         <v>48</v>
@@ -3562,45 +3515,45 @@
     </row>
     <row r="69" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>287</v>
+      </c>
+      <c r="B69" t="s">
+        <v>43</v>
+      </c>
+      <c r="C69" t="s">
+        <v>44</v>
+      </c>
+      <c r="D69" t="s">
         <v>288</v>
       </c>
-      <c r="B69" t="s">
-        <v>43</v>
-      </c>
-      <c r="C69" t="s">
-        <v>44</v>
-      </c>
-      <c r="D69" t="s">
+      <c r="J69" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="J69" t="s">
-        <v>290</v>
-      </c>
       <c r="AJ69" t="s">
         <v>48</v>
       </c>
       <c r="AO69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>290</v>
+      </c>
+      <c r="B70" t="s">
+        <v>43</v>
+      </c>
+      <c r="C70" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70" t="s">
         <v>291</v>
       </c>
-      <c r="B70" t="s">
-        <v>43</v>
-      </c>
-      <c r="C70" t="s">
-        <v>44</v>
-      </c>
-      <c r="D70" t="s">
+      <c r="J70" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="J70" t="s">
-        <v>293</v>
-      </c>
       <c r="R70" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AJ70" t="s">
         <v>48</v>
@@ -3608,22 +3561,22 @@
     </row>
     <row r="71" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>293</v>
+      </c>
+      <c r="B71" t="s">
+        <v>43</v>
+      </c>
+      <c r="C71" t="s">
+        <v>44</v>
+      </c>
+      <c r="D71" t="s">
         <v>294</v>
       </c>
-      <c r="B71" t="s">
-        <v>43</v>
-      </c>
-      <c r="C71" t="s">
-        <v>44</v>
-      </c>
-      <c r="D71" t="s">
+      <c r="J71" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="J71" t="s">
-        <v>296</v>
-      </c>
       <c r="W71" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AJ71" t="s">
         <v>48</v>
@@ -3634,7 +3587,7 @@
     </row>
     <row r="72" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B72" t="s">
         <v>43</v>
@@ -3643,16 +3596,16 @@
         <v>44</v>
       </c>
       <c r="D72" t="s">
+        <v>296</v>
+      </c>
+      <c r="J72" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="J72" t="s">
+      <c r="S72" t="s">
+        <v>177</v>
+      </c>
+      <c r="T72" t="s">
         <v>298</v>
-      </c>
-      <c r="S72" t="s">
-        <v>178</v>
-      </c>
-      <c r="T72" t="s">
-        <v>299</v>
       </c>
       <c r="AJ72" t="s">
         <v>48</v>
@@ -3660,120 +3613,120 @@
     </row>
     <row r="73" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>299</v>
+      </c>
+      <c r="B73" t="s">
+        <v>43</v>
+      </c>
+      <c r="C73" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73" t="s">
         <v>300</v>
       </c>
-      <c r="B73" t="s">
-        <v>43</v>
-      </c>
-      <c r="C73" t="s">
-        <v>44</v>
-      </c>
-      <c r="D73" t="s">
+      <c r="J73" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="J73" t="s">
-        <v>302</v>
-      </c>
       <c r="S73" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ73" t="s">
         <v>48</v>
       </c>
       <c r="AO73" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="74" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>302</v>
+      </c>
+      <c r="B74" t="s">
+        <v>43</v>
+      </c>
+      <c r="C74" t="s">
+        <v>44</v>
+      </c>
+      <c r="D74" t="s">
         <v>303</v>
       </c>
-      <c r="B74" t="s">
-        <v>43</v>
-      </c>
-      <c r="C74" t="s">
-        <v>44</v>
-      </c>
-      <c r="D74" t="s">
+      <c r="J74" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="J74" t="s">
-        <v>305</v>
-      </c>
       <c r="AJ74" t="s">
         <v>48</v>
       </c>
       <c r="AO74" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>305</v>
+      </c>
+      <c r="B75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C75" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75" t="s">
         <v>306</v>
       </c>
-      <c r="B75" t="s">
-        <v>43</v>
-      </c>
-      <c r="C75" t="s">
-        <v>44</v>
-      </c>
-      <c r="D75" t="s">
+      <c r="J75" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="J75" t="s">
-        <v>308</v>
-      </c>
       <c r="AJ75" t="s">
         <v>48</v>
       </c>
       <c r="AO75" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>237</v>
+      </c>
+      <c r="B76" t="s">
+        <v>43</v>
+      </c>
+      <c r="C76" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" t="s">
+        <v>308</v>
+      </c>
+      <c r="J76" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="R76" t="s">
+        <v>234</v>
+      </c>
+      <c r="S76" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ76" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO76" t="s">
         <v>238</v>
-      </c>
-      <c r="B76" t="s">
-        <v>43</v>
-      </c>
-      <c r="C76" t="s">
-        <v>44</v>
-      </c>
-      <c r="D76" t="s">
-        <v>309</v>
-      </c>
-      <c r="J76" t="s">
-        <v>310</v>
-      </c>
-      <c r="R76" t="s">
-        <v>235</v>
-      </c>
-      <c r="S76" t="s">
-        <v>166</v>
-      </c>
-      <c r="AJ76" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO76" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="77" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>310</v>
+      </c>
+      <c r="B77" t="s">
+        <v>43</v>
+      </c>
+      <c r="C77" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77" t="s">
         <v>311</v>
       </c>
-      <c r="B77" t="s">
-        <v>43</v>
-      </c>
-      <c r="C77" t="s">
-        <v>44</v>
-      </c>
-      <c r="D77" t="s">
+      <c r="J77" s="4" t="s">
         <v>312</v>
-      </c>
-      <c r="J77" t="s">
-        <v>313</v>
       </c>
       <c r="AJ77" t="s">
         <v>48</v>
@@ -3784,22 +3737,22 @@
     </row>
     <row r="78" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>313</v>
+      </c>
+      <c r="B78" t="s">
+        <v>43</v>
+      </c>
+      <c r="C78" t="s">
+        <v>44</v>
+      </c>
+      <c r="D78" t="s">
         <v>314</v>
       </c>
-      <c r="B78" t="s">
-        <v>43</v>
-      </c>
-      <c r="C78" t="s">
-        <v>44</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="J78" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="J78" t="s">
-        <v>316</v>
-      </c>
       <c r="L78" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AJ78" t="s">
         <v>48</v>
@@ -3810,120 +3763,120 @@
     </row>
     <row r="79" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>316</v>
+      </c>
+      <c r="B79" t="s">
+        <v>43</v>
+      </c>
+      <c r="C79" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79" t="s">
         <v>317</v>
       </c>
-      <c r="B79" t="s">
-        <v>43</v>
-      </c>
-      <c r="C79" t="s">
-        <v>44</v>
-      </c>
-      <c r="D79" t="s">
+      <c r="J79" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="J79" t="s">
-        <v>319</v>
-      </c>
       <c r="AJ79" t="s">
         <v>48</v>
       </c>
       <c r="AO79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="80" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>319</v>
+      </c>
+      <c r="B80" t="s">
+        <v>43</v>
+      </c>
+      <c r="C80" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80" t="s">
         <v>320</v>
       </c>
-      <c r="B80" t="s">
-        <v>43</v>
-      </c>
-      <c r="C80" t="s">
-        <v>44</v>
-      </c>
-      <c r="D80" t="s">
+      <c r="J80" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="J80" t="s">
-        <v>322</v>
-      </c>
       <c r="S80" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="AJ80" t="s">
         <v>48</v>
       </c>
       <c r="AO80" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>322</v>
+      </c>
+      <c r="B81" t="s">
+        <v>43</v>
+      </c>
+      <c r="C81" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" t="s">
         <v>323</v>
       </c>
-      <c r="B81" t="s">
-        <v>43</v>
-      </c>
-      <c r="C81" t="s">
-        <v>44</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="J81" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="J81" t="s">
-        <v>325</v>
-      </c>
       <c r="AJ81" t="s">
         <v>48</v>
       </c>
       <c r="AO81" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>325</v>
+      </c>
+      <c r="B82" t="s">
+        <v>43</v>
+      </c>
+      <c r="C82" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" t="s">
         <v>326</v>
       </c>
-      <c r="B82" t="s">
-        <v>43</v>
-      </c>
-      <c r="C82" t="s">
-        <v>44</v>
-      </c>
-      <c r="D82" t="s">
+      <c r="J82" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="J82" t="s">
+      <c r="R82" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ82" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO82" t="s">
         <v>328</v>
-      </c>
-      <c r="R82" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ82" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO82" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="83" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>329</v>
+      </c>
+      <c r="B83" t="s">
+        <v>43</v>
+      </c>
+      <c r="C83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83" t="s">
         <v>330</v>
       </c>
-      <c r="B83" t="s">
-        <v>43</v>
-      </c>
-      <c r="C83" t="s">
-        <v>44</v>
-      </c>
-      <c r="D83" t="s">
+      <c r="J83" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="J83" t="s">
+      <c r="L83" t="s">
         <v>332</v>
-      </c>
-      <c r="L83" t="s">
-        <v>333</v>
       </c>
       <c r="AJ83" t="s">
         <v>48</v>
@@ -3934,91 +3887,91 @@
     </row>
     <row r="84" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>333</v>
+      </c>
+      <c r="B84" t="s">
+        <v>43</v>
+      </c>
+      <c r="C84" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84" t="s">
         <v>334</v>
       </c>
-      <c r="B84" t="s">
-        <v>43</v>
-      </c>
-      <c r="C84" t="s">
-        <v>44</v>
-      </c>
-      <c r="D84" t="s">
+      <c r="J84" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="J84" t="s">
-        <v>336</v>
-      </c>
       <c r="AJ84" t="s">
         <v>48</v>
       </c>
       <c r="AO84" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>336</v>
+      </c>
+      <c r="B85" t="s">
+        <v>43</v>
+      </c>
+      <c r="C85" t="s">
+        <v>44</v>
+      </c>
+      <c r="D85" t="s">
         <v>337</v>
       </c>
-      <c r="B85" t="s">
-        <v>43</v>
-      </c>
-      <c r="C85" t="s">
-        <v>44</v>
-      </c>
-      <c r="D85" t="s">
+      <c r="J85" s="4" t="s">
         <v>338</v>
       </c>
-      <c r="J85" t="s">
-        <v>339</v>
-      </c>
       <c r="AJ85" t="s">
         <v>48</v>
       </c>
       <c r="AO85" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>339</v>
+      </c>
+      <c r="B86" t="s">
+        <v>43</v>
+      </c>
+      <c r="C86" t="s">
+        <v>44</v>
+      </c>
+      <c r="D86" t="s">
         <v>340</v>
       </c>
-      <c r="B86" t="s">
-        <v>43</v>
-      </c>
-      <c r="C86" t="s">
-        <v>44</v>
-      </c>
-      <c r="D86" t="s">
-        <v>341</v>
-      </c>
-      <c r="J86" t="s">
-        <v>339</v>
+      <c r="J86" s="4" t="s">
+        <v>338</v>
       </c>
       <c r="AJ86" t="s">
         <v>48</v>
       </c>
       <c r="AO86" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>341</v>
+      </c>
+      <c r="B87" t="s">
+        <v>43</v>
+      </c>
+      <c r="C87" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87" t="s">
         <v>342</v>
       </c>
-      <c r="B87" t="s">
-        <v>43</v>
-      </c>
-      <c r="C87" t="s">
-        <v>44</v>
-      </c>
-      <c r="D87" t="s">
+      <c r="J87" s="4" t="s">
         <v>343</v>
       </c>
-      <c r="J87" t="s">
-        <v>344</v>
-      </c>
       <c r="P87" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ87" t="s">
         <v>48</v>
@@ -4026,313 +3979,313 @@
     </row>
     <row r="88" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>344</v>
+      </c>
+      <c r="B88" t="s">
+        <v>43</v>
+      </c>
+      <c r="C88" t="s">
+        <v>44</v>
+      </c>
+      <c r="D88" t="s">
         <v>345</v>
       </c>
-      <c r="B88" t="s">
-        <v>43</v>
-      </c>
-      <c r="C88" t="s">
-        <v>44</v>
-      </c>
-      <c r="D88" t="s">
+      <c r="J88" s="4" t="s">
         <v>346</v>
       </c>
-      <c r="J88" t="s">
-        <v>347</v>
-      </c>
       <c r="AJ88" t="s">
         <v>48</v>
       </c>
       <c r="AO88" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="89" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>347</v>
+      </c>
+      <c r="B89" t="s">
+        <v>43</v>
+      </c>
+      <c r="C89" t="s">
+        <v>44</v>
+      </c>
+      <c r="D89" t="s">
         <v>348</v>
       </c>
-      <c r="B89" t="s">
-        <v>43</v>
-      </c>
-      <c r="C89" t="s">
-        <v>44</v>
-      </c>
-      <c r="D89" t="s">
+      <c r="J89" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="J89" t="s">
-        <v>350</v>
-      </c>
       <c r="AJ89" t="s">
         <v>48</v>
       </c>
       <c r="AO89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>350</v>
+      </c>
+      <c r="B90" t="s">
+        <v>43</v>
+      </c>
+      <c r="C90" t="s">
+        <v>44</v>
+      </c>
+      <c r="D90" t="s">
         <v>351</v>
       </c>
-      <c r="B90" t="s">
-        <v>43</v>
-      </c>
-      <c r="C90" t="s">
-        <v>44</v>
-      </c>
-      <c r="D90" t="s">
+      <c r="J90" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="J90" t="s">
-        <v>353</v>
-      </c>
       <c r="W90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AJ90" t="s">
         <v>48</v>
       </c>
       <c r="AO90" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="91" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>353</v>
+      </c>
+      <c r="B91" t="s">
+        <v>43</v>
+      </c>
+      <c r="C91" t="s">
+        <v>44</v>
+      </c>
+      <c r="D91" t="s">
         <v>354</v>
       </c>
-      <c r="B91" t="s">
-        <v>43</v>
-      </c>
-      <c r="C91" t="s">
-        <v>44</v>
-      </c>
-      <c r="D91" t="s">
+      <c r="J91" s="4" t="s">
         <v>355</v>
       </c>
-      <c r="J91" t="s">
-        <v>356</v>
-      </c>
       <c r="AJ91" t="s">
         <v>48</v>
       </c>
       <c r="AO91" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="92" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>356</v>
+      </c>
+      <c r="B92" t="s">
+        <v>43</v>
+      </c>
+      <c r="C92" t="s">
+        <v>44</v>
+      </c>
+      <c r="D92" t="s">
         <v>357</v>
       </c>
-      <c r="B92" t="s">
-        <v>43</v>
-      </c>
-      <c r="C92" t="s">
-        <v>44</v>
-      </c>
-      <c r="D92" t="s">
+      <c r="J92" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="J92" t="s">
-        <v>359</v>
-      </c>
       <c r="W92" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AJ92" t="s">
         <v>48</v>
       </c>
       <c r="AO92" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>359</v>
+      </c>
+      <c r="B93" t="s">
+        <v>43</v>
+      </c>
+      <c r="C93" t="s">
+        <v>44</v>
+      </c>
+      <c r="D93" t="s">
         <v>360</v>
       </c>
-      <c r="B93" t="s">
-        <v>43</v>
-      </c>
-      <c r="C93" t="s">
-        <v>44</v>
-      </c>
-      <c r="D93" t="s">
+      <c r="J93" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="J93" t="s">
-        <v>362</v>
-      </c>
       <c r="AJ93" t="s">
         <v>48</v>
       </c>
       <c r="AO93" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>362</v>
+      </c>
+      <c r="B94" t="s">
+        <v>43</v>
+      </c>
+      <c r="C94" t="s">
+        <v>44</v>
+      </c>
+      <c r="D94" t="s">
         <v>363</v>
       </c>
-      <c r="B94" t="s">
-        <v>43</v>
-      </c>
-      <c r="C94" t="s">
-        <v>44</v>
-      </c>
-      <c r="D94" t="s">
+      <c r="J94" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="J94" t="s">
-        <v>365</v>
-      </c>
       <c r="AJ94" t="s">
         <v>48</v>
       </c>
       <c r="AO94" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="95" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>365</v>
+      </c>
+      <c r="B95" t="s">
+        <v>43</v>
+      </c>
+      <c r="C95" t="s">
+        <v>44</v>
+      </c>
+      <c r="D95" t="s">
         <v>366</v>
       </c>
-      <c r="B95" t="s">
-        <v>43</v>
-      </c>
-      <c r="C95" t="s">
-        <v>44</v>
-      </c>
-      <c r="D95" t="s">
+      <c r="J95" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="J95" t="s">
-        <v>368</v>
-      </c>
       <c r="AJ95" t="s">
         <v>48</v>
       </c>
       <c r="AO95" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="96" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>368</v>
+      </c>
+      <c r="B96" t="s">
+        <v>43</v>
+      </c>
+      <c r="C96" t="s">
+        <v>44</v>
+      </c>
+      <c r="D96" t="s">
         <v>369</v>
       </c>
-      <c r="B96" t="s">
-        <v>43</v>
-      </c>
-      <c r="C96" t="s">
-        <v>44</v>
-      </c>
-      <c r="D96" t="s">
+      <c r="J96" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="J96" t="s">
-        <v>371</v>
-      </c>
       <c r="AJ96" t="s">
         <v>48</v>
       </c>
       <c r="AO96" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>371</v>
+      </c>
+      <c r="B97" t="s">
+        <v>43</v>
+      </c>
+      <c r="C97" t="s">
+        <v>44</v>
+      </c>
+      <c r="D97" t="s">
         <v>372</v>
       </c>
-      <c r="B97" t="s">
-        <v>43</v>
-      </c>
-      <c r="C97" t="s">
-        <v>44</v>
-      </c>
-      <c r="D97" t="s">
+      <c r="J97" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="J97" t="s">
-        <v>374</v>
-      </c>
       <c r="AJ97" t="s">
         <v>48</v>
       </c>
       <c r="AO97" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="98" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>374</v>
+      </c>
+      <c r="B98" t="s">
+        <v>43</v>
+      </c>
+      <c r="C98" t="s">
+        <v>44</v>
+      </c>
+      <c r="D98" t="s">
         <v>375</v>
       </c>
-      <c r="B98" t="s">
-        <v>43</v>
-      </c>
-      <c r="C98" t="s">
-        <v>44</v>
-      </c>
-      <c r="D98" t="s">
+      <c r="J98" s="4" t="s">
         <v>376</v>
       </c>
-      <c r="J98" t="s">
+      <c r="R98" t="s">
         <v>377</v>
       </c>
-      <c r="R98" t="s">
-        <v>378</v>
-      </c>
       <c r="AJ98" t="s">
         <v>48</v>
       </c>
       <c r="AO98" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="99" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>377</v>
+      </c>
+      <c r="B99" t="s">
+        <v>43</v>
+      </c>
+      <c r="C99" t="s">
+        <v>44</v>
+      </c>
+      <c r="D99" t="s">
         <v>378</v>
       </c>
-      <c r="B99" t="s">
-        <v>43</v>
-      </c>
-      <c r="C99" t="s">
-        <v>44</v>
-      </c>
-      <c r="D99" t="s">
+      <c r="J99" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="J99" t="s">
-        <v>380</v>
-      </c>
       <c r="R99" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="W99" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AJ99" t="s">
         <v>48</v>
       </c>
       <c r="AO99" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="100" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>380</v>
+      </c>
+      <c r="B100" t="s">
+        <v>43</v>
+      </c>
+      <c r="C100" t="s">
+        <v>44</v>
+      </c>
+      <c r="D100" t="s">
         <v>381</v>
       </c>
-      <c r="B100" t="s">
-        <v>43</v>
-      </c>
-      <c r="C100" t="s">
-        <v>44</v>
-      </c>
-      <c r="D100" t="s">
+      <c r="J100" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="J100" t="s">
-        <v>383</v>
-      </c>
       <c r="S100" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AJ100" t="s">
         <v>48</v>
@@ -4340,194 +4293,194 @@
     </row>
     <row r="101" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>383</v>
+      </c>
+      <c r="B101" t="s">
+        <v>43</v>
+      </c>
+      <c r="C101" t="s">
+        <v>44</v>
+      </c>
+      <c r="D101" t="s">
         <v>384</v>
       </c>
-      <c r="B101" t="s">
-        <v>43</v>
-      </c>
-      <c r="C101" t="s">
-        <v>44</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="J101" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="J101" t="s">
-        <v>386</v>
-      </c>
       <c r="AJ101" t="s">
         <v>48</v>
       </c>
       <c r="AO101" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="102" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>386</v>
+      </c>
+      <c r="B102" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" t="s">
+        <v>44</v>
+      </c>
+      <c r="D102" t="s">
         <v>387</v>
       </c>
-      <c r="B102" t="s">
-        <v>43</v>
-      </c>
-      <c r="C102" t="s">
-        <v>44</v>
-      </c>
-      <c r="D102" t="s">
+      <c r="J102" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="J102" t="s">
-        <v>389</v>
-      </c>
       <c r="AJ102" t="s">
         <v>48</v>
       </c>
       <c r="AO102" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="103" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>389</v>
+      </c>
+      <c r="B103" t="s">
+        <v>43</v>
+      </c>
+      <c r="C103" t="s">
+        <v>44</v>
+      </c>
+      <c r="D103" t="s">
         <v>390</v>
       </c>
-      <c r="B103" t="s">
-        <v>43</v>
-      </c>
-      <c r="C103" t="s">
-        <v>44</v>
-      </c>
-      <c r="D103" t="s">
+      <c r="J103" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="J103" t="s">
+      <c r="W103" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ103" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO103" t="s">
         <v>392</v>
-      </c>
-      <c r="W103" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ103" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO103" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="104" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>393</v>
+      </c>
+      <c r="B104" t="s">
+        <v>43</v>
+      </c>
+      <c r="C104" t="s">
+        <v>44</v>
+      </c>
+      <c r="D104" t="s">
         <v>394</v>
       </c>
-      <c r="B104" t="s">
-        <v>43</v>
-      </c>
-      <c r="C104" t="s">
-        <v>44</v>
-      </c>
-      <c r="D104" t="s">
+      <c r="J104" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="J104" t="s">
-        <v>396</v>
-      </c>
       <c r="AJ104" t="s">
         <v>48</v>
       </c>
       <c r="AO104" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="105" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>396</v>
+      </c>
+      <c r="B105" t="s">
+        <v>43</v>
+      </c>
+      <c r="C105" t="s">
+        <v>44</v>
+      </c>
+      <c r="D105" t="s">
         <v>397</v>
       </c>
-      <c r="B105" t="s">
-        <v>43</v>
-      </c>
-      <c r="C105" t="s">
-        <v>44</v>
-      </c>
-      <c r="D105" t="s">
+      <c r="J105" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="J105" t="s">
-        <v>399</v>
-      </c>
       <c r="AJ105" t="s">
         <v>48</v>
       </c>
       <c r="AO105" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="106" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
+        <v>399</v>
+      </c>
+      <c r="B106" t="s">
+        <v>43</v>
+      </c>
+      <c r="C106" t="s">
+        <v>44</v>
+      </c>
+      <c r="D106" t="s">
         <v>400</v>
       </c>
-      <c r="B106" t="s">
-        <v>43</v>
-      </c>
-      <c r="C106" t="s">
-        <v>44</v>
-      </c>
-      <c r="D106" t="s">
+      <c r="J106" s="4" t="s">
         <v>401</v>
       </c>
-      <c r="J106" t="s">
-        <v>402</v>
-      </c>
       <c r="AJ106" t="s">
         <v>48</v>
       </c>
       <c r="AO106" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="107" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
+        <v>402</v>
+      </c>
+      <c r="B107" t="s">
+        <v>43</v>
+      </c>
+      <c r="C107" t="s">
+        <v>44</v>
+      </c>
+      <c r="D107" t="s">
         <v>403</v>
       </c>
-      <c r="B107" t="s">
-        <v>43</v>
-      </c>
-      <c r="C107" t="s">
-        <v>44</v>
-      </c>
-      <c r="D107" t="s">
+      <c r="J107" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="J107" t="s">
-        <v>405</v>
-      </c>
       <c r="AJ107" t="s">
         <v>48</v>
       </c>
       <c r="AO107" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="108" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
+        <v>405</v>
+      </c>
+      <c r="B108" t="s">
+        <v>43</v>
+      </c>
+      <c r="C108" t="s">
+        <v>44</v>
+      </c>
+      <c r="D108" t="s">
         <v>406</v>
       </c>
-      <c r="B108" t="s">
-        <v>43</v>
-      </c>
-      <c r="C108" t="s">
-        <v>44</v>
-      </c>
-      <c r="D108" t="s">
+      <c r="J108" s="4" t="s">
         <v>407</v>
       </c>
-      <c r="J108" t="s">
-        <v>408</v>
-      </c>
       <c r="AJ108" t="s">
         <v>48</v>
       </c>
       <c r="AO108" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="109" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B109" t="s">
         <v>43</v>
@@ -4536,48 +4489,48 @@
         <v>44</v>
       </c>
       <c r="D109" t="s">
+        <v>408</v>
+      </c>
+      <c r="J109" s="4" t="s">
         <v>409</v>
       </c>
-      <c r="J109" t="s">
+      <c r="L109" t="s">
+        <v>88</v>
+      </c>
+      <c r="R109" t="s">
         <v>410</v>
       </c>
-      <c r="L109" t="s">
+      <c r="T109" t="s">
+        <v>411</v>
+      </c>
+      <c r="AJ109" t="s">
+        <v>48</v>
+      </c>
+      <c r="AO109" t="s">
         <v>89</v>
-      </c>
-      <c r="R109" t="s">
-        <v>411</v>
-      </c>
-      <c r="T109" t="s">
-        <v>412</v>
-      </c>
-      <c r="AJ109" t="s">
-        <v>48</v>
-      </c>
-      <c r="AO109" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="110" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>412</v>
+      </c>
+      <c r="B110" t="s">
+        <v>43</v>
+      </c>
+      <c r="C110" t="s">
+        <v>44</v>
+      </c>
+      <c r="D110" t="s">
         <v>413</v>
       </c>
-      <c r="B110" t="s">
-        <v>43</v>
-      </c>
-      <c r="C110" t="s">
-        <v>44</v>
-      </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>414</v>
       </c>
-      <c r="E110" t="s">
+      <c r="J110" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="J110" t="s">
-        <v>416</v>
-      </c>
       <c r="R110" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AJ110" t="s">
         <v>48</v>
@@ -4585,50 +4538,50 @@
     </row>
     <row r="111" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>416</v>
+      </c>
+      <c r="B111" t="s">
+        <v>43</v>
+      </c>
+      <c r="C111" t="s">
+        <v>44</v>
+      </c>
+      <c r="D111" t="s">
         <v>417</v>
       </c>
-      <c r="B111" t="s">
-        <v>43</v>
-      </c>
-      <c r="C111" t="s">
-        <v>44</v>
-      </c>
-      <c r="D111" t="s">
+      <c r="J111" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="J111" t="s">
-        <v>419</v>
-      </c>
       <c r="AJ111" t="s">
         <v>48</v>
       </c>
       <c r="AO111" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="112" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>419</v>
+      </c>
+      <c r="B112" t="s">
+        <v>43</v>
+      </c>
+      <c r="C112" t="s">
+        <v>44</v>
+      </c>
+      <c r="D112" t="s">
         <v>420</v>
       </c>
-      <c r="B112" t="s">
-        <v>43</v>
-      </c>
-      <c r="C112" t="s">
-        <v>44</v>
-      </c>
-      <c r="D112" t="s">
+      <c r="J112" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="J112" t="s">
+      <c r="AI112" t="s">
         <v>422</v>
-      </c>
-      <c r="AI112" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="113" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B113" t="s">
         <v>43</v>
@@ -4637,16 +4590,16 @@
         <v>44</v>
       </c>
       <c r="D113" t="s">
+        <v>423</v>
+      </c>
+      <c r="J113" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="J113" t="s">
+      <c r="Q113" t="s">
+        <v>341</v>
+      </c>
+      <c r="T113" t="s">
         <v>425</v>
-      </c>
-      <c r="Q113" t="s">
-        <v>342</v>
-      </c>
-      <c r="T113" t="s">
-        <v>426</v>
       </c>
       <c r="AJ113" t="s">
         <v>48</v>
@@ -4654,19 +4607,19 @@
     </row>
     <row r="114" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>426</v>
+      </c>
+      <c r="B114" t="s">
+        <v>43</v>
+      </c>
+      <c r="C114" t="s">
+        <v>44</v>
+      </c>
+      <c r="D114" t="s">
         <v>427</v>
       </c>
-      <c r="B114" t="s">
-        <v>43</v>
-      </c>
-      <c r="C114" t="s">
-        <v>44</v>
-      </c>
-      <c r="D114" t="s">
+      <c r="J114" s="4" t="s">
         <v>428</v>
-      </c>
-      <c r="J114" t="s">
-        <v>429</v>
       </c>
       <c r="W114" t="s">
         <v>47</v>
@@ -4680,123 +4633,52 @@
     </row>
     <row r="115" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>429</v>
+      </c>
+      <c r="B115" t="s">
+        <v>43</v>
+      </c>
+      <c r="C115" t="s">
+        <v>44</v>
+      </c>
+      <c r="D115" t="s">
         <v>430</v>
       </c>
-      <c r="B115" t="s">
-        <v>43</v>
-      </c>
-      <c r="C115" t="s">
-        <v>44</v>
-      </c>
-      <c r="D115" t="s">
+      <c r="J115" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="J115" t="s">
-        <v>432</v>
-      </c>
       <c r="AJ115" t="s">
         <v>48</v>
       </c>
       <c r="AO115" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J30" r:id="rId1" xr:uid="{5D7A6E1D-005A-4356-9DEB-92E97E8666C6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B1" t="s">
         <v>433</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>434</v>
-      </c>
-      <c r="C1" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>436</v>
-      </c>
-      <c r="B2" t="s">
-        <v>437</v>
-      </c>
-      <c r="C2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>439</v>
-      </c>
-      <c r="B3" t="s">
-        <v>437</v>
-      </c>
-      <c r="C3" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>440</v>
-      </c>
-      <c r="B4" t="s">
-        <v>437</v>
-      </c>
-      <c r="C4" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" t="s">
-        <v>437</v>
-      </c>
-      <c r="C5" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B6" t="s">
-        <v>437</v>
-      </c>
-      <c r="C6" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" t="s">
-        <v>437</v>
-      </c>
-      <c r="C7" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B8" t="s">
-        <v>437</v>
-      </c>
-      <c r="C8" t="s">
-        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -4806,128 +4688,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B1" t="s">
         <v>433</v>
       </c>
-      <c r="B1" t="s">
-        <v>434</v>
-      </c>
       <c r="C1" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>436</v>
-      </c>
-      <c r="B2" t="s">
-        <v>443</v>
-      </c>
-      <c r="C2" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>439</v>
-      </c>
-      <c r="B3" t="s">
-        <v>445</v>
-      </c>
-      <c r="C3" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>440</v>
-      </c>
-      <c r="B4" t="s">
-        <v>445</v>
-      </c>
-      <c r="C4" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>446</v>
-      </c>
-      <c r="B5" t="s">
-        <v>447</v>
-      </c>
-      <c r="C5" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>449</v>
-      </c>
-      <c r="B6" t="s">
-        <v>447</v>
-      </c>
-      <c r="C6" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>450</v>
-      </c>
-      <c r="B7" t="s">
-        <v>451</v>
-      </c>
-      <c r="C7" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>453</v>
-      </c>
-      <c r="B8" t="s">
-        <v>454</v>
-      </c>
-      <c r="C8" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>456</v>
-      </c>
-      <c r="B9" t="s">
-        <v>457</v>
-      </c>
-      <c r="C9" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>458</v>
-      </c>
-      <c r="B10" t="s">
-        <v>459</v>
-      </c>
-      <c r="C10" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>460</v>
-      </c>
-      <c r="B11" t="s">
-        <v>459</v>
-      </c>
-      <c r="C11" t="s">
-        <v>455</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>